<commit_message>
05.2: store Loss Limit tool_id as text; 05.3 and 05.4: align with manuscript, correct cooldown values and convergent figures
</commit_message>
<xml_diff>
--- a/materials/05_implementation_architectures/asb_framework_05_2_nl_implementation_architecture.xlsx
+++ b/materials/05_implementation_architectures/asb_framework_05_2_nl_implementation_architecture.xlsx
@@ -1153,7 +1153,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="74" t="inlineStr">
         <is>
@@ -1271,7 +1270,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="74" t="inlineStr">
         <is>
@@ -1631,7 +1629,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="74" t="inlineStr">
         <is>
@@ -1674,7 +1671,6 @@
       <c r="C33" s="56" t="n"/>
       <c r="D33" s="57" t="n"/>
     </row>
-    <row r="34"/>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="80" t="inlineStr">
         <is>
@@ -1724,7 +1720,6 @@
       <c r="C38" s="56" t="n"/>
       <c r="D38" s="57" t="n"/>
     </row>
-    <row r="39"/>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="80" t="inlineStr">
         <is>
@@ -1802,7 +1797,6 @@
       <c r="C45" s="56" t="n"/>
       <c r="D45" s="57" t="n"/>
     </row>
-    <row r="46"/>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="80" t="inlineStr">
         <is>
@@ -1922,7 +1916,6 @@
       <c r="C55" s="56" t="n"/>
       <c r="D55" s="57" t="n"/>
     </row>
-    <row r="56"/>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="80" t="inlineStr">
         <is>
@@ -1986,7 +1979,6 @@
       <c r="C61" s="56" t="n"/>
       <c r="D61" s="57" t="n"/>
     </row>
-    <row r="62"/>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="80" t="inlineStr">
         <is>
@@ -2036,7 +2028,6 @@
       <c r="C66" s="56" t="n"/>
       <c r="D66" s="57" t="n"/>
     </row>
-    <row r="67"/>
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="80" t="inlineStr">
         <is>
@@ -2072,7 +2063,6 @@
       <c r="C70" s="56" t="n"/>
       <c r="D70" s="57" t="n"/>
     </row>
-    <row r="71"/>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="80" t="inlineStr">
         <is>
@@ -2150,7 +2140,6 @@
       <c r="C77" s="56" t="n"/>
       <c r="D77" s="57" t="n"/>
     </row>
-    <row r="78"/>
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="80" t="inlineStr">
         <is>
@@ -2214,7 +2203,6 @@
       <c r="C83" s="56" t="n"/>
       <c r="D83" s="57" t="n"/>
     </row>
-    <row r="84"/>
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="80" t="inlineStr">
         <is>
@@ -4270,8 +4258,10 @@
           <t>loss_limit</t>
         </is>
       </c>
-      <c r="B35" s="77" t="n">
-        <v>1.1</v>
+      <c r="B35" s="77" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
       <c r="C35" s="77" t="inlineStr">
         <is>
@@ -4335,8 +4325,10 @@
           <t>loss_limit</t>
         </is>
       </c>
-      <c r="B36" s="79" t="n">
-        <v>1.1</v>
+      <c r="B36" s="79" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
       <c r="C36" s="79" t="inlineStr">
         <is>
@@ -4398,8 +4390,10 @@
           <t>loss_limit</t>
         </is>
       </c>
-      <c r="B37" s="77" t="n">
-        <v>1.1</v>
+      <c r="B37" s="77" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
       <c r="C37" s="77" t="inlineStr">
         <is>
@@ -4463,8 +4457,10 @@
           <t>loss_limit</t>
         </is>
       </c>
-      <c r="B38" s="79" t="n">
-        <v>1.1</v>
+      <c r="B38" s="79" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
       <c r="C38" s="79" t="inlineStr">
         <is>
@@ -4526,8 +4522,10 @@
           <t>loss_limit</t>
         </is>
       </c>
-      <c r="B39" s="77" t="n">
-        <v>1.1</v>
+      <c r="B39" s="77" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
       <c r="C39" s="77" t="inlineStr">
         <is>
@@ -4591,8 +4589,10 @@
           <t>loss_limit</t>
         </is>
       </c>
-      <c r="B40" s="79" t="n">
-        <v>1.1</v>
+      <c r="B40" s="79" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
       <c r="C40" s="79" t="inlineStr">
         <is>
@@ -4654,8 +4654,10 @@
           <t>loss_limit</t>
         </is>
       </c>
-      <c r="B41" s="77" t="n">
-        <v>1.1</v>
+      <c r="B41" s="77" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
       <c r="C41" s="77" t="inlineStr">
         <is>
@@ -4717,8 +4719,10 @@
           <t>loss_limit</t>
         </is>
       </c>
-      <c r="B42" s="79" t="n">
-        <v>1.1</v>
+      <c r="B42" s="79" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
       </c>
       <c r="C42" s="79" t="inlineStr">
         <is>

</xml_diff>